<commit_message>
release: finalize EconoCausal v1.0.0 deliverables and audit trail
</commit_message>
<xml_diff>
--- a/05_Final_Deliverables/Model_Evaluation_Report.xlsx
+++ b/05_Final_Deliverables/Model_Evaluation_Report.xlsx
@@ -500,7 +500,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -911,7 +910,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1462,7 +1460,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1627,7 +1624,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1917,7 +1913,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2299,7 +2294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="82" customWidth="1" min="1" max="1"/>
@@ -2324,7 +2319,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2482,6 +2476,38 @@
       <c r="F8" s="5" t="inlineStr">
         <is>
           <t>PASS — Common Support Holds</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Model-Based Residual Permutation Diagnostic</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>+14.22%</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>[-2.12%, +2.02%]</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Permutation null test</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>p = 0.0020 (p &lt; 0.05)</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>PASS — Invariant to Permutation</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2547,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2847,7 +2872,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2898,12 +2922,12 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3 Safe</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -2913,12 +2937,12 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2 Quarantined</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>100% VERIFIED PASS</t>
+          <t>1 Live Pass (2 WDAC Blocked)</t>
         </is>
       </c>
     </row>
@@ -2935,12 +2959,12 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -2955,7 +2979,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>100% VERIFIED PASS</t>
+          <t>100% LIVE VERIFIED PASS (23.8s)</t>
         </is>
       </c>
     </row>
@@ -2972,12 +2996,12 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>14 Hist.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -2992,7 +3016,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>100% VERIFIED PASS</t>
+          <t>100% Hist. Pass (WDAC Constrained in L8)</t>
         </is>
       </c>
     </row>
@@ -3009,12 +3033,12 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>34</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>33</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -3029,7 +3053,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>100% VERIFIED PASS</t>
+          <t>33 LIVE PASS, 1 WDAC Blocked (65.5s)</t>
         </is>
       </c>
     </row>
@@ -3066,29 +3090,29 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>100% VERIFIED PASS (543ms)</t>
+          <t>100% LIVE VERIFIED PASS (2.22s)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Complete End-to-End Test Suite</t>
+          <t>Automated Test Inventory</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>All 5 Repositories</t>
+          <t>Active Repository Codebase</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>66 Defined</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>64 Safe</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -3098,12 +3122,12 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2 Quarantined</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>100% VERIFIED PASS (Zero Failures)</t>
+          <t>49 Live Pass, 18 WDAC, 2 Quarantined</t>
         </is>
       </c>
     </row>

</xml_diff>